<commit_message>
Remove colored avatar material from public experience
</commit_message>
<xml_diff>
--- a/content/个人作品网站内容管理.xlsx
+++ b/content/个人作品网站内容管理.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网站方向" sheetId="1" r:id="R30045ca6ab324422"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面规划" sheetId="2" r:id="R5f699ef879994ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作品库" sheetId="3" r:id="Rd69ceccb86e0456d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="多语言文案" sheetId="4" r:id="Rc26641c4228a40ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="素材库" sheetId="5" r:id="Rcfee10e8db784aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新说明" sheetId="6" r:id="Rc9be0bc9728742fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网站方向" sheetId="1" r:id="R8069dad672884936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面规划" sheetId="2" r:id="Re3831f7009c34796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="作品库" sheetId="3" r:id="Reb1c082f46ec4ff3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="多语言文案" sheetId="4" r:id="Rf9eae749308e49a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="素材库" sheetId="5" r:id="Rad2df99643674f5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="更新说明" sheetId="6" r:id="R523249ac6a324823"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -622,7 +622,7 @@
         <x:v>首页默认头像效果</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
-        <x:v>原始 / 大理石 / 镜面，三选一</x:v>
+        <x:v>大理石 / 镜面；彩色原始版停用，未来探索其他材质</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
         <x:v>待选择</x:v>
@@ -650,7 +650,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcdd13324d544aa4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95bcd1f801784c1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -949,16 +949,16 @@
         <x:v>/about</x:v>
       </x:c>
       <x:c r="D15" s="10" t="str">
-        <x:v>保留</x:v>
+        <x:v>隐藏</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="F15" s="10" t="str">
-        <x:v>原始贴图、跟随、蓝光、文字避让与波纹</x:v>
+        <x:v>彩色贴图效果不采用；保留编号作为历史记录</x:v>
       </x:c>
       <x:c r="G15" s="9" t="str">
-        <x:v>已上线；后续路径待统一</x:v>
+        <x:v>已从公开入口移除；/about 现为大理石别名</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="56" customHeight="1">
@@ -978,10 +978,10 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="F16" s="10" t="str">
-        <x:v>大理石与局部彩色显露</x:v>
+        <x:v>黑色大理石与局部单色石墨材质变化</x:v>
       </x:c>
       <x:c r="G16" s="9" t="str">
-        <x:v>已上线</x:v>
+        <x:v>已上线；当前为探索版本，后续继续尝试其他材质</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="56" customHeight="1">
@@ -1084,7 +1084,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c1332d6b4a843e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bd7df11191f4456"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1322,7 +1322,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refa592444ae44e66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1031995f3af40ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2419,7 +2419,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ff64e9feae494b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d45718e99c54ab4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2712,7 +2712,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b003fbff916417f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69ad9d66a4f64c78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2885,7 +2885,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc5bb47e83ac4038"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d873092523485f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>